<commit_message>
Add new food spots to the shared list.
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\OneDrive\Documents\Cursor Projects\food-spot-selector\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9412421F-B8C3-49A3-AD76-04498C9F40DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF0B9289-60D3-4B3F-98B7-F16D02FE9BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="275">
   <si>
     <t>Place</t>
   </si>
@@ -100,9 +100,6 @@
     <t>Lai Cai Ke Kou Mian Clarke Quay</t>
   </si>
   <si>
-    <t>ENEN Ke Kou Main Orchard Towers</t>
-  </si>
-  <si>
     <t>Ming Fa Fishball Noodles</t>
   </si>
   <si>
@@ -806,6 +803,48 @@
   </si>
   <si>
     <t>Ramen, Noodles</t>
+  </si>
+  <si>
+    <t>ENEN Ke Kou Main</t>
+  </si>
+  <si>
+    <t>East, Central</t>
+  </si>
+  <si>
+    <t>Phuket Town Mookata</t>
+  </si>
+  <si>
+    <t>Tom Yam Mama</t>
+  </si>
+  <si>
+    <t>Kiap Kiap Chicken Club &amp; Bar</t>
+  </si>
+  <si>
+    <t>Fried Chicken</t>
+  </si>
+  <si>
+    <t>Le Cheng Kampong Hainanese Chicken Rice</t>
+  </si>
+  <si>
+    <t>The Soup Expert</t>
+  </si>
+  <si>
+    <t>Nanjing Impressions</t>
+  </si>
+  <si>
+    <t>Longjing Restaurant</t>
+  </si>
+  <si>
+    <t>THREE BOWLS 来三碗</t>
+  </si>
+  <si>
+    <t>Kolo Mee, Noodles</t>
+  </si>
+  <si>
+    <t>Huiwei Duck Claypot</t>
+  </si>
+  <si>
+    <t>Duck Claypot</t>
   </si>
 </sst>
 </file>
@@ -1129,18 +1168,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H152"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:H160"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.921875" style="1" customWidth="1"/>
-    <col min="2" max="3" width="29.69140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
+    <col min="2" max="3" width="29.7265625" style="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" customWidth="1"/>
-    <col min="5" max="6" width="15.15234375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.4609375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="27.61328125" style="1" customWidth="1"/>
+    <col min="5" max="6" width="15.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.6328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1163,7 +1202,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1186,7 +1225,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1209,7 +1248,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1232,7 +1271,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -1255,7 +1294,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="58.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="58.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1278,7 +1317,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -1301,7 +1340,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
@@ -1324,9 +1363,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>261</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>8</v>
@@ -1344,12 +1383,12 @@
         <v>21</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>8</v>
@@ -1370,15 +1409,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D11" s="1">
         <v>10</v>
@@ -1393,15 +1432,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="D12" s="1">
         <v>18</v>
@@ -1416,15 +1455,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="D13" s="1">
         <v>12</v>
@@ -1439,12 +1478,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="D14" s="1">
         <v>12</v>
@@ -1459,12 +1498,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="1">
         <v>12</v>
@@ -1479,12 +1518,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D16" s="1">
         <v>17</v>
@@ -1499,15 +1538,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="D17" s="1">
         <v>17</v>
@@ -1522,12 +1561,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="D18" s="1">
         <v>11</v>
@@ -1539,12 +1578,12 @@
         <v>21</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>8</v>
@@ -1565,9 +1604,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>8</v>
@@ -1582,18 +1621,18 @@
         <v>21</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="D21" s="1">
         <v>12</v>
@@ -1608,15 +1647,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="D22" s="1">
         <v>11</v>
@@ -1628,15 +1667,15 @@
         <v>21</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A23" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="B23" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D23" s="1">
         <v>12</v>
@@ -1648,18 +1687,18 @@
         <v>21</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="D24" s="1">
         <v>12</v>
@@ -1671,15 +1710,15 @@
         <v>21</v>
       </c>
       <c r="G24" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A25" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="B25" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D25" s="1">
         <v>12</v>
@@ -1694,15 +1733,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D26" s="1">
         <v>7</v>
@@ -1717,15 +1756,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D27" s="1">
         <v>8</v>
@@ -1740,15 +1779,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="D28" s="1">
         <v>12</v>
@@ -1763,9 +1802,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>8</v>
@@ -1783,15 +1822,15 @@
         <v>18</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="D30" s="1">
         <v>11</v>
@@ -1806,9 +1845,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="43.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" ht="43.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>8</v>
@@ -1829,9 +1868,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>8</v>
@@ -1849,15 +1888,15 @@
         <v>21</v>
       </c>
       <c r="G32" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="B33" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>24</v>
@@ -1872,18 +1911,18 @@
         <v>21</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="D34" s="1">
         <v>11</v>
@@ -1898,15 +1937,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="D35" s="1">
         <v>15</v>
@@ -1921,9 +1960,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>8</v>
@@ -1944,15 +1983,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="D37" s="1">
         <v>10</v>
@@ -1964,15 +2003,15 @@
         <v>21</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="D38" s="1">
         <v>18</v>
@@ -1981,18 +2020,18 @@
         <v>23</v>
       </c>
       <c r="F38" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A39" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D39" s="1">
         <v>12</v>
@@ -2007,12 +2046,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D40" s="1">
         <v>12</v>
@@ -2027,15 +2066,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="D41" s="2">
         <v>12</v>
@@ -2047,15 +2086,15 @@
         <v>21</v>
       </c>
       <c r="G41" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A42" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="B42" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D42" s="1">
         <v>12</v>
@@ -2067,18 +2106,18 @@
         <v>21</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="D43" s="1">
         <v>9</v>
@@ -2093,15 +2132,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="D44" s="1">
         <v>10</v>
@@ -2113,18 +2152,18 @@
         <v>21</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D45" s="1">
         <v>10</v>
@@ -2139,12 +2178,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D46" s="1">
         <v>16</v>
@@ -2159,15 +2198,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="D47" s="1">
         <v>11</v>
@@ -2182,15 +2221,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B48" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="D48" s="1">
         <v>18</v>
@@ -2205,15 +2244,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="D49" s="1">
         <v>11</v>
@@ -2225,18 +2264,18 @@
         <v>18</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B50" t="s">
         <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D50">
         <v>10</v>
@@ -2248,18 +2287,18 @@
         <v>21</v>
       </c>
       <c r="G50" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>98</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
         <v>99</v>
-      </c>
-      <c r="B51" t="s">
-        <v>8</v>
-      </c>
-      <c r="C51" t="s">
-        <v>100</v>
       </c>
       <c r="D51">
         <v>17</v>
@@ -2268,21 +2307,21 @@
         <v>0</v>
       </c>
       <c r="F51" t="s">
+        <v>100</v>
+      </c>
+      <c r="G51" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>101</v>
       </c>
-      <c r="G51" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A52" t="s">
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
         <v>102</v>
-      </c>
-      <c r="B52" t="s">
-        <v>8</v>
-      </c>
-      <c r="C52" t="s">
-        <v>103</v>
       </c>
       <c r="D52">
         <v>12</v>
@@ -2297,15 +2336,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
+        <v>103</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
         <v>104</v>
-      </c>
-      <c r="B53" t="s">
-        <v>8</v>
-      </c>
-      <c r="C53" t="s">
-        <v>105</v>
       </c>
       <c r="D53">
         <v>11</v>
@@ -2317,18 +2356,18 @@
         <v>18</v>
       </c>
       <c r="G53" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" t="s">
         <v>106</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>107</v>
-      </c>
-      <c r="C54" t="s">
-        <v>108</v>
       </c>
       <c r="D54">
         <v>7</v>
@@ -2337,15 +2376,15 @@
         <v>14</v>
       </c>
       <c r="F54" t="s">
+        <v>108</v>
+      </c>
+      <c r="G54" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>109</v>
-      </c>
-      <c r="G54" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A55" t="s">
-        <v>110</v>
       </c>
       <c r="B55" t="s">
         <v>8</v>
@@ -2360,15 +2399,15 @@
         <v>23</v>
       </c>
       <c r="F55" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G55" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" t="s">
         <v>8</v>
@@ -2386,15 +2425,15 @@
         <v>10</v>
       </c>
       <c r="G56" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B57" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D57">
         <v>11</v>
@@ -2409,15 +2448,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
+        <v>112</v>
+      </c>
+      <c r="B58" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58" t="s">
         <v>113</v>
-      </c>
-      <c r="B58" t="s">
-        <v>8</v>
-      </c>
-      <c r="C58" t="s">
-        <v>114</v>
       </c>
       <c r="D58">
         <v>5</v>
@@ -2432,15 +2471,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
+        <v>114</v>
+      </c>
+      <c r="B59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" t="s">
         <v>115</v>
-      </c>
-      <c r="B59" t="s">
-        <v>8</v>
-      </c>
-      <c r="C59" t="s">
-        <v>116</v>
       </c>
       <c r="D59">
         <v>6</v>
@@ -2452,12 +2491,12 @@
         <v>21</v>
       </c>
       <c r="G59" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B60" t="s">
         <v>8</v>
@@ -2478,15 +2517,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" t="s">
         <v>118</v>
-      </c>
-      <c r="B61" t="s">
-        <v>8</v>
-      </c>
-      <c r="C61" t="s">
-        <v>119</v>
       </c>
       <c r="D61">
         <v>10</v>
@@ -2501,15 +2540,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B62" t="s">
         <v>8</v>
       </c>
       <c r="C62" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D62">
         <v>17</v>
@@ -2524,15 +2563,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
+        <v>120</v>
+      </c>
+      <c r="B63" t="s">
+        <v>106</v>
+      </c>
+      <c r="C63" t="s">
         <v>121</v>
-      </c>
-      <c r="B63" t="s">
-        <v>107</v>
-      </c>
-      <c r="C63" t="s">
-        <v>122</v>
       </c>
       <c r="D63">
         <v>11</v>
@@ -2547,9 +2586,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B64" t="s">
         <v>8</v>
@@ -2564,21 +2603,21 @@
         <v>20</v>
       </c>
       <c r="F64" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G64" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B65" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C65" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D65">
         <v>11</v>
@@ -2593,15 +2632,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B66" t="s">
         <v>8</v>
       </c>
       <c r="C66" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D66">
         <v>9</v>
@@ -2616,15 +2655,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
+        <v>125</v>
+      </c>
+      <c r="B67" t="s">
+        <v>106</v>
+      </c>
+      <c r="C67" t="s">
         <v>126</v>
-      </c>
-      <c r="B67" t="s">
-        <v>107</v>
-      </c>
-      <c r="C67" t="s">
-        <v>127</v>
       </c>
       <c r="D67">
         <v>11</v>
@@ -2639,9 +2678,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B68" t="s">
         <v>8</v>
@@ -2662,9 +2701,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B69" t="s">
         <v>8</v>
@@ -2679,21 +2718,21 @@
         <v>13</v>
       </c>
       <c r="F69" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G69" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
+        <v>129</v>
+      </c>
+      <c r="B70" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
         <v>130</v>
-      </c>
-      <c r="B70" t="s">
-        <v>8</v>
-      </c>
-      <c r="C70" t="s">
-        <v>131</v>
       </c>
       <c r="D70">
         <v>8</v>
@@ -2708,15 +2747,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B71" t="s">
         <v>8</v>
       </c>
       <c r="C71" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D71">
         <v>12</v>
@@ -2725,21 +2764,21 @@
         <v>18</v>
       </c>
       <c r="F71" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G71" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
+        <v>132</v>
+      </c>
+      <c r="B72" t="s">
+        <v>8</v>
+      </c>
+      <c r="C72" t="s">
         <v>133</v>
-      </c>
-      <c r="B72" t="s">
-        <v>8</v>
-      </c>
-      <c r="C72" t="s">
-        <v>134</v>
       </c>
       <c r="D72">
         <v>7</v>
@@ -2754,15 +2793,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B73" t="s">
         <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D73">
         <v>10</v>
@@ -2777,12 +2816,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
+        <v>135</v>
+      </c>
+      <c r="B74" t="s">
         <v>136</v>
-      </c>
-      <c r="B74" t="s">
-        <v>137</v>
       </c>
       <c r="D74">
         <v>12</v>
@@ -2794,18 +2833,18 @@
         <v>21</v>
       </c>
       <c r="G74" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B75" t="s">
         <v>8</v>
       </c>
       <c r="C75" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D75">
         <v>11</v>
@@ -2820,15 +2859,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B76" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C76" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D76">
         <v>9</v>
@@ -2843,15 +2882,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B77" t="s">
         <v>8</v>
       </c>
       <c r="C77" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D77">
         <v>8</v>
@@ -2860,21 +2899,21 @@
         <v>19</v>
       </c>
       <c r="F77" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G77" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
+        <v>140</v>
+      </c>
+      <c r="B78" t="s">
+        <v>8</v>
+      </c>
+      <c r="C78" t="s">
         <v>141</v>
-      </c>
-      <c r="B78" t="s">
-        <v>8</v>
-      </c>
-      <c r="C78" t="s">
-        <v>142</v>
       </c>
       <c r="D78">
         <v>8</v>
@@ -2889,15 +2928,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D79">
         <v>12</v>
@@ -2912,15 +2951,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B80" t="s">
         <v>8</v>
       </c>
       <c r="C80" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D80">
         <v>12</v>
@@ -2929,21 +2968,21 @@
         <v>20</v>
       </c>
       <c r="F80" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G80" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
+        <v>144</v>
+      </c>
+      <c r="B81" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" t="s">
         <v>145</v>
-      </c>
-      <c r="B81" t="s">
-        <v>8</v>
-      </c>
-      <c r="C81" t="s">
-        <v>146</v>
       </c>
       <c r="D81">
         <v>8</v>
@@ -2958,9 +2997,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B82" t="s">
         <v>8</v>
@@ -2978,18 +3017,18 @@
         <v>21</v>
       </c>
       <c r="G82" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B83" t="s">
         <v>8</v>
       </c>
       <c r="C83" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D83">
         <v>11</v>
@@ -3004,15 +3043,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B84" t="s">
         <v>8</v>
       </c>
       <c r="C84" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D84">
         <v>9</v>
@@ -3021,21 +3060,21 @@
         <v>14</v>
       </c>
       <c r="F84" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G84" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
+        <v>149</v>
+      </c>
+      <c r="B85" t="s">
+        <v>8</v>
+      </c>
+      <c r="C85" t="s">
         <v>150</v>
-      </c>
-      <c r="B85" t="s">
-        <v>8</v>
-      </c>
-      <c r="C85" t="s">
-        <v>151</v>
       </c>
       <c r="D85">
         <v>10</v>
@@ -3050,15 +3089,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B86" t="s">
         <v>8</v>
       </c>
       <c r="C86" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D86">
         <v>10</v>
@@ -3067,15 +3106,15 @@
         <v>14</v>
       </c>
       <c r="F86" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G86" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B87" t="s">
         <v>8</v>
@@ -3090,15 +3129,15 @@
         <v>20</v>
       </c>
       <c r="F87" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G87" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B88" t="s">
         <v>8</v>
@@ -3110,41 +3149,41 @@
         <v>15</v>
       </c>
       <c r="F88" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G88" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
+        <v>154</v>
+      </c>
+      <c r="B89" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89" t="s">
         <v>155</v>
       </c>
-      <c r="B89" t="s">
-        <v>8</v>
-      </c>
-      <c r="C89" t="s">
+      <c r="D89">
+        <v>11</v>
+      </c>
+      <c r="E89">
+        <v>21</v>
+      </c>
+      <c r="F89" t="s">
+        <v>237</v>
+      </c>
+      <c r="G89" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>156</v>
       </c>
-      <c r="D89">
-        <v>11</v>
-      </c>
-      <c r="E89">
-        <v>21</v>
-      </c>
-      <c r="F89" t="s">
-        <v>238</v>
-      </c>
-      <c r="G89" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A90" t="s">
+      <c r="B90" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="D90">
         <v>12</v>
@@ -3159,15 +3198,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B91" t="s">
         <v>8</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D91">
         <v>8</v>
@@ -3176,21 +3215,21 @@
         <v>15</v>
       </c>
       <c r="F91" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G91" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B92" t="s">
         <v>8</v>
       </c>
       <c r="C92" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D92">
         <v>8</v>
@@ -3199,21 +3238,21 @@
         <v>15</v>
       </c>
       <c r="F92" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G92" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
+        <v>160</v>
+      </c>
+      <c r="B93" t="s">
+        <v>8</v>
+      </c>
+      <c r="C93" t="s">
         <v>161</v>
-      </c>
-      <c r="B93" t="s">
-        <v>8</v>
-      </c>
-      <c r="C93" t="s">
-        <v>162</v>
       </c>
       <c r="D93">
         <v>11</v>
@@ -3222,15 +3261,15 @@
         <v>20</v>
       </c>
       <c r="F93" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G93" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B94" t="s">
         <v>8</v>
@@ -3248,18 +3287,18 @@
         <v>21</v>
       </c>
       <c r="G94" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
+        <v>163</v>
+      </c>
+      <c r="B95" t="s">
+        <v>8</v>
+      </c>
+      <c r="C95" t="s">
         <v>164</v>
-      </c>
-      <c r="B95" t="s">
-        <v>8</v>
-      </c>
-      <c r="C95" t="s">
-        <v>165</v>
       </c>
       <c r="D95">
         <v>9</v>
@@ -3274,15 +3313,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
+        <v>165</v>
+      </c>
+      <c r="B96" t="s">
+        <v>8</v>
+      </c>
+      <c r="C96" t="s">
         <v>166</v>
-      </c>
-      <c r="B96" t="s">
-        <v>8</v>
-      </c>
-      <c r="C96" t="s">
-        <v>167</v>
       </c>
       <c r="D96">
         <v>7</v>
@@ -3297,15 +3336,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
+        <v>167</v>
+      </c>
+      <c r="B97" t="s">
+        <v>8</v>
+      </c>
+      <c r="C97" t="s">
         <v>168</v>
-      </c>
-      <c r="B97" t="s">
-        <v>8</v>
-      </c>
-      <c r="C97" t="s">
-        <v>169</v>
       </c>
       <c r="D97">
         <v>8</v>
@@ -3320,12 +3359,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B98" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D98">
         <v>18</v>
@@ -3340,15 +3379,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B99" t="s">
         <v>8</v>
       </c>
       <c r="C99" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D99">
         <v>7</v>
@@ -3363,15 +3402,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
+        <v>171</v>
+      </c>
+      <c r="B100" t="s">
         <v>172</v>
       </c>
-      <c r="B100" t="s">
+      <c r="C100" t="s">
         <v>173</v>
-      </c>
-      <c r="C100" t="s">
-        <v>174</v>
       </c>
       <c r="D100">
         <v>11</v>
@@ -3386,15 +3425,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B101" t="s">
         <v>8</v>
       </c>
       <c r="C101" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D101">
         <v>9</v>
@@ -3409,15 +3448,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B102" t="s">
         <v>8</v>
       </c>
       <c r="C102" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D102">
         <v>12</v>
@@ -3432,12 +3471,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
+        <v>176</v>
+      </c>
+      <c r="B103" t="s">
         <v>177</v>
-      </c>
-      <c r="B103" t="s">
-        <v>178</v>
       </c>
       <c r="D103">
         <v>18</v>
@@ -3452,15 +3491,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B104" t="s">
         <v>8</v>
       </c>
       <c r="C104" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D104">
         <v>11</v>
@@ -3475,15 +3514,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B105" t="s">
         <v>8</v>
       </c>
       <c r="C105" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D105">
         <v>8</v>
@@ -3498,15 +3537,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B106" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C106" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D106">
         <v>11</v>
@@ -3521,15 +3560,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
+        <v>181</v>
+      </c>
+      <c r="B107" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107" t="s">
         <v>182</v>
-      </c>
-      <c r="B107" t="s">
-        <v>8</v>
-      </c>
-      <c r="C107" t="s">
-        <v>183</v>
       </c>
       <c r="D107">
         <v>6</v>
@@ -3544,15 +3583,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
+        <v>183</v>
+      </c>
+      <c r="B108" t="s">
+        <v>8</v>
+      </c>
+      <c r="C108" t="s">
         <v>184</v>
-      </c>
-      <c r="B108" t="s">
-        <v>8</v>
-      </c>
-      <c r="C108" t="s">
-        <v>185</v>
       </c>
       <c r="D108">
         <v>12</v>
@@ -3561,21 +3600,21 @@
         <v>22</v>
       </c>
       <c r="F108" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G108" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
+        <v>185</v>
+      </c>
+      <c r="B109" t="s">
+        <v>8</v>
+      </c>
+      <c r="C109" t="s">
         <v>186</v>
-      </c>
-      <c r="B109" t="s">
-        <v>8</v>
-      </c>
-      <c r="C109" t="s">
-        <v>187</v>
       </c>
       <c r="D109">
         <v>15</v>
@@ -3584,21 +3623,21 @@
         <v>21</v>
       </c>
       <c r="F109" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G109" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
+        <v>187</v>
+      </c>
+      <c r="B110" t="s">
+        <v>8</v>
+      </c>
+      <c r="C110" t="s">
         <v>188</v>
-      </c>
-      <c r="B110" t="s">
-        <v>8</v>
-      </c>
-      <c r="C110" t="s">
-        <v>189</v>
       </c>
       <c r="D110">
         <v>7</v>
@@ -3613,9 +3652,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B111" t="s">
         <v>8</v>
@@ -3636,12 +3675,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B112" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D112">
         <v>11</v>
@@ -3656,15 +3695,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B113" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C113" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D113">
         <v>10</v>
@@ -3679,15 +3718,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B114" t="s">
         <v>8</v>
       </c>
       <c r="C114" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D114">
         <v>11</v>
@@ -3702,15 +3741,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
+        <v>193</v>
+      </c>
+      <c r="B115" t="s">
+        <v>8</v>
+      </c>
+      <c r="C115" t="s">
         <v>194</v>
-      </c>
-      <c r="B115" t="s">
-        <v>8</v>
-      </c>
-      <c r="C115" t="s">
-        <v>195</v>
       </c>
       <c r="D115">
         <v>10</v>
@@ -3722,18 +3761,18 @@
         <v>18</v>
       </c>
       <c r="G115" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B116" t="s">
         <v>8</v>
       </c>
       <c r="C116" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D116">
         <v>10</v>
@@ -3748,15 +3787,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B117" t="s">
         <v>8</v>
       </c>
       <c r="C117" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D117">
         <v>12</v>
@@ -3765,21 +3804,21 @@
         <v>21</v>
       </c>
       <c r="F117" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G117" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B118" t="s">
         <v>8</v>
       </c>
       <c r="C118" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D118">
         <v>6</v>
@@ -3788,21 +3827,21 @@
         <v>15</v>
       </c>
       <c r="F118" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G118" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B119" t="s">
         <v>8</v>
       </c>
       <c r="C119" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D119">
         <v>6</v>
@@ -3817,15 +3856,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B120" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C120" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D120">
         <v>8</v>
@@ -3834,21 +3873,21 @@
         <v>19</v>
       </c>
       <c r="F120" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G120" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B121" t="s">
         <v>8</v>
       </c>
       <c r="C121" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D121">
         <v>12</v>
@@ -3863,15 +3902,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B122" t="s">
         <v>8</v>
       </c>
       <c r="C122" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D122">
         <v>10</v>
@@ -3883,18 +3922,18 @@
         <v>18</v>
       </c>
       <c r="G122" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B123" t="s">
         <v>8</v>
       </c>
       <c r="C123" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D123">
         <v>11</v>
@@ -3906,18 +3945,18 @@
         <v>21</v>
       </c>
       <c r="G123" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B124" t="s">
         <v>8</v>
       </c>
       <c r="C124" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D124">
         <v>15</v>
@@ -3932,15 +3971,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B125" t="s">
         <v>8</v>
       </c>
       <c r="C125" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D125">
         <v>9</v>
@@ -3949,21 +3988,21 @@
         <v>19</v>
       </c>
       <c r="F125" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G125" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B126" t="s">
         <v>8</v>
       </c>
       <c r="C126" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D126">
         <v>9</v>
@@ -3978,15 +4017,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B127" t="s">
         <v>8</v>
       </c>
       <c r="C127" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D127">
         <v>10</v>
@@ -4001,15 +4040,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B128" t="s">
         <v>8</v>
       </c>
       <c r="C128" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D128">
         <v>10</v>
@@ -4024,9 +4063,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B129" t="s">
         <v>8</v>
@@ -4041,21 +4080,21 @@
         <v>20</v>
       </c>
       <c r="F129" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G129" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B130" t="s">
         <v>8</v>
       </c>
       <c r="C130" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D130">
         <v>9</v>
@@ -4070,9 +4109,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B131" t="s">
         <v>8</v>
@@ -4093,12 +4132,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B132" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D132">
         <v>12</v>
@@ -4113,15 +4152,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B133" t="s">
+        <v>172</v>
+      </c>
+      <c r="C133" t="s">
         <v>173</v>
-      </c>
-      <c r="C133" t="s">
-        <v>174</v>
       </c>
       <c r="D133">
         <v>11</v>
@@ -4133,12 +4172,12 @@
         <v>21</v>
       </c>
       <c r="G133" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B134" t="s">
         <v>8</v>
@@ -4159,12 +4198,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B135" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D135">
         <v>11</v>
@@ -4179,12 +4218,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B136" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D136">
         <v>11</v>
@@ -4199,12 +4238,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
+        <v>215</v>
+      </c>
+      <c r="B137" t="s">
         <v>216</v>
-      </c>
-      <c r="B137" t="s">
-        <v>217</v>
       </c>
       <c r="D137">
         <v>11</v>
@@ -4219,15 +4258,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
+        <v>217</v>
+      </c>
+      <c r="B138" t="s">
+        <v>8</v>
+      </c>
+      <c r="C138" t="s">
         <v>218</v>
-      </c>
-      <c r="B138" t="s">
-        <v>8</v>
-      </c>
-      <c r="C138" t="s">
-        <v>219</v>
       </c>
       <c r="D138">
         <v>16</v>
@@ -4236,18 +4275,18 @@
         <v>20</v>
       </c>
       <c r="F138" t="s">
+        <v>219</v>
+      </c>
+      <c r="G138" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
         <v>220</v>
       </c>
-      <c r="G138" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A139" t="s">
-        <v>221</v>
-      </c>
       <c r="B139" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D139">
         <v>11</v>
@@ -4262,15 +4301,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B140" t="s">
         <v>8</v>
       </c>
       <c r="C140" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D140">
         <v>5</v>
@@ -4285,15 +4324,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B141" t="s">
         <v>8</v>
       </c>
       <c r="C141" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D141">
         <v>7</v>
@@ -4308,15 +4347,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B142" t="s">
         <v>8</v>
       </c>
       <c r="C142" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D142">
         <v>11</v>
@@ -4331,15 +4370,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B143" t="s">
         <v>8</v>
       </c>
       <c r="C143" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D143">
         <v>11</v>
@@ -4354,15 +4393,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C144" s="1" t="s">
         <v>226</v>
-      </c>
-      <c r="B144" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C144" s="1" t="s">
-        <v>227</v>
       </c>
       <c r="D144" s="1">
         <v>6</v>
@@ -4374,18 +4413,18 @@
         <v>10</v>
       </c>
       <c r="G144" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C145" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="B145" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C145" s="1" t="s">
-        <v>229</v>
       </c>
       <c r="D145" s="1">
         <v>11</v>
@@ -4397,18 +4436,18 @@
         <v>21</v>
       </c>
       <c r="G145" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B146" t="s">
         <v>8</v>
       </c>
       <c r="C146" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D146">
         <v>6</v>
@@ -4417,21 +4456,21 @@
         <v>14</v>
       </c>
       <c r="F146" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G146" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
+        <v>230</v>
+      </c>
+      <c r="B147" t="s">
+        <v>8</v>
+      </c>
+      <c r="C147" t="s">
         <v>231</v>
-      </c>
-      <c r="B147" t="s">
-        <v>8</v>
-      </c>
-      <c r="C147" t="s">
-        <v>232</v>
       </c>
       <c r="D147">
         <v>8</v>
@@ -4443,18 +4482,18 @@
         <v>14</v>
       </c>
       <c r="G147" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
+        <v>232</v>
+      </c>
+      <c r="B148" t="s">
+        <v>8</v>
+      </c>
+      <c r="C148" t="s">
         <v>233</v>
-      </c>
-      <c r="B148" t="s">
-        <v>8</v>
-      </c>
-      <c r="C148" t="s">
-        <v>234</v>
       </c>
       <c r="D148">
         <v>8</v>
@@ -4463,21 +4502,21 @@
         <v>17</v>
       </c>
       <c r="F148" t="s">
+        <v>234</v>
+      </c>
+      <c r="G148" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
         <v>235</v>
       </c>
-      <c r="G148" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A149" t="s">
-        <v>236</v>
-      </c>
       <c r="B149" t="s">
         <v>8</v>
       </c>
       <c r="C149" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D149">
         <v>7</v>
@@ -4486,21 +4525,21 @@
         <v>14</v>
       </c>
       <c r="F149" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G149" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B150" t="s">
         <v>8</v>
       </c>
       <c r="C150" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D150">
         <v>8</v>
@@ -4509,21 +4548,21 @@
         <v>23</v>
       </c>
       <c r="F150" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G150" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
+        <v>238</v>
+      </c>
+      <c r="B151" t="s">
+        <v>8</v>
+      </c>
+      <c r="C151" t="s">
         <v>239</v>
-      </c>
-      <c r="B151" t="s">
-        <v>8</v>
-      </c>
-      <c r="C151" t="s">
-        <v>240</v>
       </c>
       <c r="D151">
         <v>11</v>
@@ -4535,18 +4574,18 @@
         <v>18</v>
       </c>
       <c r="G151" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C152" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="B152" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>261</v>
       </c>
       <c r="D152" s="1">
         <v>11</v>
@@ -4561,7 +4600,183 @@
         <v>11</v>
       </c>
     </row>
+    <row r="153" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A153" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D153" s="1">
+        <v>12</v>
+      </c>
+      <c r="E153" s="1">
+        <v>1</v>
+      </c>
+      <c r="F153" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G153" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A154" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="D154" s="1">
+        <v>18</v>
+      </c>
+      <c r="E154" s="1">
+        <v>2</v>
+      </c>
+      <c r="F154" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G154" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A155" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D155" s="1">
+        <v>10</v>
+      </c>
+      <c r="E155" s="1">
+        <v>0</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G155" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A156" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D156" s="1">
+        <v>12</v>
+      </c>
+      <c r="E156" s="1">
+        <v>21</v>
+      </c>
+      <c r="F156" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G156" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A157" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D157" s="1">
+        <v>11</v>
+      </c>
+      <c r="E157" s="1">
+        <v>21</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G157" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A158" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D158" s="1">
+        <v>11</v>
+      </c>
+      <c r="E158" s="1">
+        <v>22</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G158" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A159" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D159" s="1">
+        <v>13</v>
+      </c>
+      <c r="E159" s="1">
+        <v>21</v>
+      </c>
+      <c r="F159" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G159" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A160" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D160" s="1">
+        <v>12</v>
+      </c>
+      <c r="E160" s="1">
+        <v>22</v>
+      </c>
+      <c r="F160" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G160" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync the expanded food spot list from Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF0B9289-60D3-4B3F-98B7-F16D02FE9BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA2C3E1-F575-4F8D-B74E-C965E2336BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="290">
   <si>
     <t>Place</t>
   </si>
@@ -845,6 +845,51 @@
   </si>
   <si>
     <t>Duck Claypot</t>
+  </si>
+  <si>
+    <t>Zenryoku Izakaya</t>
+  </si>
+  <si>
+    <t>Izakaya</t>
+  </si>
+  <si>
+    <t>Ramen Story</t>
+  </si>
+  <si>
+    <t>Ramen Soshiji</t>
+  </si>
+  <si>
+    <t>Enishi Ramen</t>
+  </si>
+  <si>
+    <t>Ume San 100</t>
+  </si>
+  <si>
+    <t>Uma Haus</t>
+  </si>
+  <si>
+    <t>Bari Uma</t>
+  </si>
+  <si>
+    <t>Gunkee Claypot</t>
+  </si>
+  <si>
+    <t>Fatty Ox Famous Kitchen</t>
+  </si>
+  <si>
+    <t>Hong Kong</t>
+  </si>
+  <si>
+    <t>No. 25 Minced Meat Noodle</t>
+  </si>
+  <si>
+    <t>Sat, Sun, Wed</t>
+  </si>
+  <si>
+    <t>Yamamoto's Hamburg</t>
+  </si>
+  <si>
+    <t>Hamburg</t>
   </si>
 </sst>
 </file>
@@ -1168,7 +1213,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H171"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
@@ -1485,6 +1530,9 @@
       <c r="B14" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="C14" s="1" t="s">
+        <v>276</v>
+      </c>
       <c r="D14" s="1">
         <v>12</v>
       </c>
@@ -1505,6 +1553,9 @@
       <c r="B15" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="C15" s="1" t="s">
+        <v>276</v>
+      </c>
       <c r="D15" s="1">
         <v>12</v>
       </c>
@@ -1720,6 +1771,9 @@
       <c r="B25" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="C25" s="1" t="s">
+        <v>276</v>
+      </c>
       <c r="D25" s="1">
         <v>12</v>
       </c>
@@ -2096,6 +2150,9 @@
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="C42" s="1" t="s">
+        <v>276</v>
+      </c>
       <c r="D42" s="1">
         <v>12</v>
       </c>
@@ -4772,6 +4829,256 @@
         <v>21</v>
       </c>
       <c r="G160" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A161" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="D161" s="1">
+        <v>12</v>
+      </c>
+      <c r="E161" s="1">
+        <v>0</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G161" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A162" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D162" s="1">
+        <v>11</v>
+      </c>
+      <c r="E162" s="1">
+        <v>21</v>
+      </c>
+      <c r="F162" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G162" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A163" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D163" s="1">
+        <v>12</v>
+      </c>
+      <c r="E163" s="1">
+        <v>4</v>
+      </c>
+      <c r="F163" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G163" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A164" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D164" s="1">
+        <v>11</v>
+      </c>
+      <c r="E164" s="1">
+        <v>21</v>
+      </c>
+      <c r="F164" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G164" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A165" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D165" s="1">
+        <v>12</v>
+      </c>
+      <c r="E165" s="1">
+        <v>22</v>
+      </c>
+      <c r="F165" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G165" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A166" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D166" s="1">
+        <v>10</v>
+      </c>
+      <c r="E166" s="1">
+        <v>20</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G166" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A167" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D167" s="1">
+        <v>11</v>
+      </c>
+      <c r="E167" s="1">
+        <v>22</v>
+      </c>
+      <c r="F167" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G167" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A168" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D168" s="1">
+        <v>11</v>
+      </c>
+      <c r="E168" s="1">
+        <v>23</v>
+      </c>
+      <c r="F168" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G168" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A169" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D169" s="1">
+        <v>8</v>
+      </c>
+      <c r="E169" s="1">
+        <v>14</v>
+      </c>
+      <c r="F169" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G169" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A170" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D170" s="1">
+        <v>8</v>
+      </c>
+      <c r="E170" s="1">
+        <v>14</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="G170" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A171" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D171" s="1">
+        <v>11</v>
+      </c>
+      <c r="E171" s="1">
+        <v>21</v>
+      </c>
+      <c r="F171" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G171" s="1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>